<commit_message>
Regenerate fabrication outputs and add impedance/fab reference docs
Update gerbers, BOM, positions, and netlist to match the latest PCB
edits, including the new User Drawings layer. Add the JLCPCB
impedance calculation screenshot and a one-page fabrication guide for
reference.
</commit_message>
<xml_diff>
--- a/production/USB_PCIE_Board.xlsx
+++ b/production/USB_PCIE_Board.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3353ad593722afaa/Ibrahim_Files/Education/Embedded_Systems/KiCAD/Projects/USB_PCIE_Board/production/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="104" documentId="8_{96CBFA76-3FEB-47DD-A241-B7C6FD43C22C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B0BC2351-07EC-4216-B02C-932367DC7BA9}"/>
+  <xr:revisionPtr revIDLastSave="122" documentId="8_{96CBFA76-3FEB-47DD-A241-B7C6FD43C22C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B9DAE0AB-2CCD-4D96-B811-56900C04C5BB}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{A24AAC1F-CDCF-4533-BD40-8D8E523E9E7A}"/>
   </bookViews>
@@ -595,18 +595,6 @@
     <t>60 Ohms @ 100 MHz 1 Power Line Ferrite Bead 0805 (2012 Metric) 3.5A 20mOhm</t>
   </si>
   <si>
-    <t>J1</t>
-  </si>
-  <si>
-    <t>Bus_PCI_Express_x1</t>
-  </si>
-  <si>
-    <t>Connector_PCBEdge:BUS_PCIexpress_x1</t>
-  </si>
-  <si>
-    <t>PCI Express bus connector x1</t>
-  </si>
-  <si>
     <t>J2,J3,J4,J5</t>
   </si>
   <si>
@@ -1331,6 +1319,18 @@
   </si>
   <si>
     <t>22 µF ±20% 6.3V Ceramic Capacitor X5R 0603 (1608 Metric)</t>
+  </si>
+  <si>
+    <t>C108081</t>
+  </si>
+  <si>
+    <t>10pF</t>
+  </si>
+  <si>
+    <t>9pF Load Capacitance</t>
+  </si>
+  <si>
+    <t>Replacement</t>
   </si>
 </sst>
 </file>
@@ -1473,7 +1473,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="36">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1659,6 +1659,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.89999084444715716"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="10">
     <border>
@@ -1820,7 +1832,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1841,6 +1853,27 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="34" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="35" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -1888,7 +1921,10 @@
     <cellStyle name="Total" xfId="17" builtinId="25" customBuiltin="1"/>
     <cellStyle name="Warning Text" xfId="14" builtinId="11" customBuiltin="1"/>
   </cellStyles>
-  <dxfs count="15">
+  <dxfs count="16">
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1959,22 +1995,23 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{03075DB7-5C33-4021-9682-326B2CA55FA2}" name="Table1" displayName="Table1" ref="A1:M59" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13">
-  <autoFilter ref="A1:M59" xr:uid="{03075DB7-5C33-4021-9682-326B2CA55FA2}"/>
-  <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{ABB7BF1E-0ECF-4418-B445-86C7390E5CBD}" name="Reference" dataDxfId="12"/>
-    <tableColumn id="2" xr3:uid="{27AF76F6-B452-4F87-825E-29AFB005CC6C}" name="Qty" dataDxfId="11"/>
-    <tableColumn id="3" xr3:uid="{396D6705-5060-41F8-B89A-AC140A5EA8E4}" name="Value" dataDxfId="10"/>
-    <tableColumn id="4" xr3:uid="{2934CB77-92B1-4DDA-B4B3-3F65E5E44735}" name="Footprint" dataDxfId="9"/>
-    <tableColumn id="5" xr3:uid="{F967E4F8-6D3F-4563-ABC8-56EA22398015}" name="Manufacturer" dataDxfId="8"/>
-    <tableColumn id="6" xr3:uid="{3EF329C5-0DFE-4F6B-84B4-03F2871CCEA4}" name="DigiKey Part #" dataDxfId="7"/>
-    <tableColumn id="7" xr3:uid="{480BDE52-5B28-4AE4-ABEB-C2DE8D79EFAB}" name="LCSC Part #" dataDxfId="6"/>
-    <tableColumn id="8" xr3:uid="{7FD11529-55C3-431F-8C9D-37172549B9E9}" name="Manufacturer Part #" dataDxfId="5"/>
-    <tableColumn id="9" xr3:uid="{AB4E976D-D26E-403F-A05C-ADFB3FFFA186}" name="Package" dataDxfId="4"/>
-    <tableColumn id="10" xr3:uid="{41135254-03D5-4824-85F2-B7D08CA1293B}" name="Tolerance" dataDxfId="3"/>
-    <tableColumn id="11" xr3:uid="{C1269622-4EC4-47A0-8D75-393BC186EF8C}" name="Voltage Rating" dataDxfId="2"/>
-    <tableColumn id="12" xr3:uid="{424F9A46-1E5C-4331-AC7F-CBEEC7504959}" name="Current Rating" dataDxfId="1"/>
-    <tableColumn id="13" xr3:uid="{15A46D8F-FE12-4506-BC08-8979886D0D5E}" name="Description" dataDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{03075DB7-5C33-4021-9682-326B2CA55FA2}" name="Table1" displayName="Table1" ref="A1:N58" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
+  <autoFilter ref="A1:N58" xr:uid="{03075DB7-5C33-4021-9682-326B2CA55FA2}"/>
+  <tableColumns count="14">
+    <tableColumn id="1" xr3:uid="{ABB7BF1E-0ECF-4418-B445-86C7390E5CBD}" name="Reference" dataDxfId="13"/>
+    <tableColumn id="2" xr3:uid="{27AF76F6-B452-4F87-825E-29AFB005CC6C}" name="Qty" dataDxfId="12"/>
+    <tableColumn id="3" xr3:uid="{396D6705-5060-41F8-B89A-AC140A5EA8E4}" name="Value" dataDxfId="11"/>
+    <tableColumn id="4" xr3:uid="{2934CB77-92B1-4DDA-B4B3-3F65E5E44735}" name="Footprint" dataDxfId="10"/>
+    <tableColumn id="5" xr3:uid="{F967E4F8-6D3F-4563-ABC8-56EA22398015}" name="Manufacturer" dataDxfId="9"/>
+    <tableColumn id="6" xr3:uid="{3EF329C5-0DFE-4F6B-84B4-03F2871CCEA4}" name="DigiKey Part #" dataDxfId="8"/>
+    <tableColumn id="7" xr3:uid="{480BDE52-5B28-4AE4-ABEB-C2DE8D79EFAB}" name="LCSC Part #" dataDxfId="7"/>
+    <tableColumn id="8" xr3:uid="{7FD11529-55C3-431F-8C9D-37172549B9E9}" name="Manufacturer Part #" dataDxfId="6"/>
+    <tableColumn id="9" xr3:uid="{AB4E976D-D26E-403F-A05C-ADFB3FFFA186}" name="Package" dataDxfId="5"/>
+    <tableColumn id="10" xr3:uid="{41135254-03D5-4824-85F2-B7D08CA1293B}" name="Tolerance" dataDxfId="4"/>
+    <tableColumn id="11" xr3:uid="{C1269622-4EC4-47A0-8D75-393BC186EF8C}" name="Voltage Rating" dataDxfId="3"/>
+    <tableColumn id="12" xr3:uid="{424F9A46-1E5C-4331-AC7F-CBEEC7504959}" name="Current Rating" dataDxfId="2"/>
+    <tableColumn id="13" xr3:uid="{15A46D8F-FE12-4506-BC08-8979886D0D5E}" name="Description" dataDxfId="1"/>
+    <tableColumn id="14" xr3:uid="{2A2F499D-D1B5-42A2-A5F2-FF5F7EAB8704}" name="Replacement" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2297,7 +2334,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8901302B-2098-47CD-A4E9-60248238156D}">
-  <dimension ref="A1:M59"/>
+  <dimension ref="A1:N58"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="41.28515625" style="1" customWidth="1"/>
@@ -2313,10 +2350,11 @@
     <col min="11" max="11" width="15.7109375" style="2" customWidth="1"/>
     <col min="12" max="12" width="15.5703125" style="2" customWidth="1"/>
     <col min="13" max="13" width="118.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="9.140625" style="1"/>
+    <col min="14" max="14" width="20.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -2356,84 +2394,91 @@
       <c r="M1" s="5" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
+      <c r="N1" s="6" t="s">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="9">
         <v>17</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="F2" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H2" s="1" t="s">
+      <c r="H2" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="10" t="s">
+        <v>414</v>
+      </c>
+      <c r="J2" s="11">
+        <v>0.1</v>
+      </c>
+      <c r="K2" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="L2" s="9"/>
+      <c r="M2" s="8" t="s">
         <v>418</v>
       </c>
-      <c r="J2" s="4">
+      <c r="N2" s="9"/>
+    </row>
+    <row r="3" spans="1:14" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" s="9">
+        <v>19</v>
+      </c>
+      <c r="C3" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F3" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="G3" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" s="10" t="s">
+        <v>414</v>
+      </c>
+      <c r="J3" s="11">
         <v>0.1</v>
       </c>
-      <c r="K2" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="B3" s="2">
-        <v>19</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>418</v>
-      </c>
-      <c r="J3" s="4">
-        <v>0.1</v>
-      </c>
-      <c r="K3" s="2" t="s">
+      <c r="K3" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="M3" s="1" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="L3" s="9"/>
+      <c r="M3" s="8" t="s">
+        <v>419</v>
+      </c>
+      <c r="N3" s="9"/>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>26</v>
       </c>
@@ -2459,7 +2504,7 @@
         <v>32</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>419</v>
+        <v>415</v>
       </c>
       <c r="J4" s="4">
         <v>0.1</v>
@@ -2468,83 +2513,91 @@
         <v>33</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="N4" s="2"/>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="13">
         <v>2</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="H5" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="I5" s="3" t="s">
-        <v>418</v>
-      </c>
-      <c r="K5" s="2" t="s">
+      <c r="I5" s="14" t="s">
+        <v>414</v>
+      </c>
+      <c r="J5" s="13"/>
+      <c r="K5" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="M5" s="1" t="s">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="L5" s="13"/>
+      <c r="M5" s="12" t="s">
+        <v>421</v>
+      </c>
+      <c r="N5" s="2" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="9">
         <v>6</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="D6" s="1" t="s">
+      <c r="D6" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="F6" s="1" t="s">
+      <c r="F6" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G6" s="8" t="s">
         <v>45</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="H6" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="I6" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="J6" s="4">
+      <c r="I6" s="10" t="s">
+        <v>416</v>
+      </c>
+      <c r="J6" s="11">
         <v>0.1</v>
       </c>
-      <c r="K6" s="2" t="s">
+      <c r="K6" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="M6" s="1" t="s">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="L6" s="9"/>
+      <c r="M6" s="8" t="s">
+        <v>422</v>
+      </c>
+      <c r="N6" s="9"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>47</v>
       </c>
@@ -2561,16 +2614,16 @@
         <v>18</v>
       </c>
       <c r="F7" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>48</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>49</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>50</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>419</v>
+        <v>415</v>
       </c>
       <c r="J7" s="4">
         <v>0.1</v>
@@ -2579,10 +2632,11 @@
         <v>40</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+        <v>423</v>
+      </c>
+      <c r="N7" s="2"/>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>51</v>
       </c>
@@ -2617,10 +2671,11 @@
         <v>33</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+        <v>424</v>
+      </c>
+      <c r="N8" s="2"/>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>56</v>
       </c>
@@ -2655,10 +2710,11 @@
         <v>62</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>429</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+        <v>425</v>
+      </c>
+      <c r="N9" s="2"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>63</v>
       </c>
@@ -2690,10 +2746,11 @@
         <v>40</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>430</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+        <v>426</v>
+      </c>
+      <c r="N10" s="2"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>71</v>
       </c>
@@ -2725,10 +2782,11 @@
         <v>40</v>
       </c>
       <c r="M11" s="1" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+        <v>427</v>
+      </c>
+      <c r="N11" s="2"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>78</v>
       </c>
@@ -2763,10 +2821,11 @@
         <v>40</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>432</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+        <v>428</v>
+      </c>
+      <c r="N12" s="2"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>83</v>
       </c>
@@ -2792,7 +2851,7 @@
         <v>87</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
       <c r="J13" s="4">
         <v>0.1</v>
@@ -2801,10 +2860,11 @@
         <v>40</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+        <v>429</v>
+      </c>
+      <c r="N13" s="2"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>88</v>
       </c>
@@ -2830,7 +2890,7 @@
         <v>92</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
       <c r="J14" s="4">
         <v>0.05</v>
@@ -2839,10 +2899,11 @@
         <v>40</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>434</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+        <v>430</v>
+      </c>
+      <c r="N14" s="2"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>93</v>
       </c>
@@ -2877,10 +2938,11 @@
         <v>99</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+        <v>431</v>
+      </c>
+      <c r="N15" s="2"/>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>100</v>
       </c>
@@ -2906,7 +2968,7 @@
         <v>103</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>419</v>
+        <v>415</v>
       </c>
       <c r="J16" s="4">
         <v>0.2</v>
@@ -2915,10 +2977,11 @@
         <v>104</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+        <v>432</v>
+      </c>
+      <c r="N16" s="2"/>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>105</v>
       </c>
@@ -2952,8 +3015,9 @@
       <c r="M17" s="1" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N17" s="2"/>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>113</v>
       </c>
@@ -2982,13 +3046,14 @@
         <v>119</v>
       </c>
       <c r="K18" s="2" t="s">
-        <v>421</v>
+        <v>417</v>
       </c>
       <c r="M18" s="1" t="s">
         <v>120</v>
       </c>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N18" s="2"/>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>121</v>
       </c>
@@ -3019,8 +3084,9 @@
       <c r="M19" s="1" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N19" s="2"/>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>129</v>
       </c>
@@ -3051,8 +3117,9 @@
       <c r="M20" s="1" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N20" s="2"/>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>137</v>
       </c>
@@ -3083,8 +3150,9 @@
       <c r="M21" s="1" t="s">
         <v>143</v>
       </c>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N21" s="2"/>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>144</v>
       </c>
@@ -3121,8 +3189,9 @@
       <c r="M22" s="1" t="s">
         <v>152</v>
       </c>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N22" s="2"/>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>153</v>
       </c>
@@ -3148,7 +3217,7 @@
         <v>158</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>420</v>
+        <v>416</v>
       </c>
       <c r="K23" s="2" t="s">
         <v>159</v>
@@ -3156,8 +3225,9 @@
       <c r="M23" s="1" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N23" s="2"/>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>161</v>
       </c>
@@ -3183,7 +3253,7 @@
         <v>165</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>420</v>
+        <v>416</v>
       </c>
       <c r="K24" s="2" t="s">
         <v>159</v>
@@ -3191,8 +3261,9 @@
       <c r="M24" s="1" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N24" s="2"/>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>167</v>
       </c>
@@ -3218,7 +3289,7 @@
         <v>172</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>420</v>
+        <v>416</v>
       </c>
       <c r="K25" s="2" t="s">
         <v>173</v>
@@ -3226,8 +3297,9 @@
       <c r="M25" s="1" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N25" s="2"/>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>175</v>
       </c>
@@ -3253,7 +3325,7 @@
         <v>181</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>419</v>
+        <v>415</v>
       </c>
       <c r="K26" s="2" t="s">
         <v>182</v>
@@ -3264,8 +3336,9 @@
       <c r="M26" s="1" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N26" s="2"/>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>185</v>
       </c>
@@ -3291,557 +3364,603 @@
         <v>186</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>420</v>
+        <v>416</v>
       </c>
       <c r="M27" s="1" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N27" s="2"/>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>191</v>
       </c>
       <c r="B28" s="2">
+        <v>4</v>
+      </c>
+      <c r="C28" s="1">
+        <v>484050001</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="H28" s="1">
+        <v>484050001</v>
+      </c>
+      <c r="M28" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="N28" s="2"/>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="B29" s="2">
         <v>1</v>
       </c>
-      <c r="C28" s="1" t="s">
-        <v>192</v>
-      </c>
-      <c r="D28" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="M28" s="1" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
-        <v>195</v>
-      </c>
-      <c r="B29" s="2">
-        <v>4</v>
-      </c>
-      <c r="C29" s="1">
-        <v>484050001</v>
+      <c r="C29" s="1" t="s">
+        <v>198</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>199</v>
+        <v>180</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="G29" s="1" t="s">
-        <v>198</v>
-      </c>
-      <c r="H29" s="1">
-        <v>484050001</v>
+        <v>201</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="L29" s="2" t="s">
+        <v>203</v>
       </c>
       <c r="M29" s="1" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+        <v>204</v>
+      </c>
+      <c r="N29" s="2"/>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="B30" s="2">
         <v>1</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>180</v>
+        <v>60</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="G30" s="1" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="H30" s="1" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="L30" s="2" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="M30" s="1" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+        <v>212</v>
+      </c>
+      <c r="N30" s="2"/>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="B31" s="2">
         <v>1</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>60</v>
+        <v>38</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="G31" s="1" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>214</v>
+        <v>218</v>
+      </c>
+      <c r="I31" s="3">
+        <v>1008</v>
       </c>
       <c r="L31" s="2" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="M31" s="1" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+        <v>220</v>
+      </c>
+      <c r="N31" s="2"/>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="B32" s="2">
         <v>1</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>38</v>
+        <v>134</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="G32" s="1" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="H32" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="I32" s="3">
-        <v>1008</v>
-      </c>
-      <c r="L32" s="2" t="s">
-        <v>223</v>
+      <c r="I32" s="3" t="s">
+        <v>226</v>
       </c>
       <c r="M32" s="1" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+        <v>227</v>
+      </c>
+      <c r="N32" s="2"/>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="B33" s="2">
         <v>1</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>134</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="G33" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="H33" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="H33" s="1" t="s">
+      <c r="I33" s="3" t="s">
         <v>226</v>
       </c>
-      <c r="I33" s="3" t="s">
-        <v>230</v>
-      </c>
       <c r="M33" s="1" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+        <v>232</v>
+      </c>
+      <c r="N33" s="2"/>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B34" s="2">
         <v>1</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="F34" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="H34" s="1" t="s">
         <v>234</v>
       </c>
-      <c r="G34" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="H34" s="1" t="s">
-        <v>233</v>
-      </c>
       <c r="I34" s="3" t="s">
-        <v>230</v>
+        <v>238</v>
+      </c>
+      <c r="L34" s="2" t="s">
+        <v>239</v>
       </c>
       <c r="M34" s="1" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+        <v>240</v>
+      </c>
+      <c r="N34" s="2"/>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="B35" s="2">
         <v>1</v>
       </c>
       <c r="C35" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>245</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="I35" s="3" t="s">
         <v>238</v>
       </c>
-      <c r="D35" s="1" t="s">
-        <v>239</v>
-      </c>
-      <c r="E35" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="F35" s="1" t="s">
-        <v>240</v>
-      </c>
-      <c r="G35" s="1" t="s">
-        <v>241</v>
-      </c>
-      <c r="H35" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="I35" s="3" t="s">
-        <v>242</v>
+      <c r="K35" s="2" t="s">
+        <v>247</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="M35" s="1" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+        <v>249</v>
+      </c>
+      <c r="N35" s="2"/>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="B36" s="2">
+        <v>5</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>253</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="H36" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="I36" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="M36" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="N36" s="2"/>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
+        <v>257</v>
+      </c>
+      <c r="B37" s="2">
+        <v>12</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="H37" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="I37" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="J37" s="4">
+        <v>0.05</v>
+      </c>
+      <c r="M37" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="N37" s="2"/>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="B38" s="2">
+        <v>2</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="H38" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="I38" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="J38" s="4">
+        <v>0.01</v>
+      </c>
+      <c r="M38" s="1" t="s">
+        <v>269</v>
+      </c>
+      <c r="N38" s="2"/>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="B39" s="2">
         <v>1</v>
       </c>
-      <c r="C36" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="D36" s="1" t="s">
-        <v>247</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>250</v>
-      </c>
-      <c r="F36" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="G36" s="1" t="s">
-        <v>249</v>
-      </c>
-      <c r="H36" s="1" t="s">
-        <v>246</v>
-      </c>
-      <c r="I36" s="3" t="s">
-        <v>242</v>
-      </c>
-      <c r="K36" s="2" t="s">
-        <v>251</v>
-      </c>
-      <c r="L36" s="2" t="s">
-        <v>252</v>
-      </c>
-      <c r="M36" s="1" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A37" s="1" t="s">
-        <v>254</v>
-      </c>
-      <c r="B37" s="2">
-        <v>5</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>255</v>
-      </c>
-      <c r="D37" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="E37" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="F37" s="1" t="s">
-        <v>257</v>
-      </c>
-      <c r="G37" s="1" t="s">
-        <v>258</v>
-      </c>
-      <c r="H37" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="I37" s="3" t="s">
-        <v>419</v>
-      </c>
-      <c r="M37" s="1" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A38" s="1" t="s">
-        <v>261</v>
-      </c>
-      <c r="B38" s="2">
-        <v>12</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>262</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>256</v>
-      </c>
-      <c r="E38" s="1" t="s">
-        <v>265</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>263</v>
-      </c>
-      <c r="G38" s="1" t="s">
-        <v>264</v>
-      </c>
-      <c r="H38" s="1" t="s">
-        <v>266</v>
-      </c>
-      <c r="I38" s="3" t="s">
-        <v>419</v>
-      </c>
-      <c r="J38" s="4">
-        <v>0.05</v>
-      </c>
-      <c r="M38" s="1" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A39" s="1" t="s">
-        <v>268</v>
-      </c>
-      <c r="B39" s="2">
-        <v>2</v>
-      </c>
       <c r="C39" s="1" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>256</v>
+        <v>272</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>18</v>
+        <v>68</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="G39" s="1" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="I39" s="3" t="s">
-        <v>419</v>
+        <v>414</v>
       </c>
       <c r="J39" s="4">
         <v>0.01</v>
       </c>
       <c r="M39" s="1" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
+        <v>276</v>
+      </c>
+      <c r="N39" s="2"/>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="B40" s="2">
         <v>1</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="E40" s="1" t="s">
         <v>68</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="G40" s="1" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="I40" s="3" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
       <c r="J40" s="4">
         <v>0.01</v>
       </c>
       <c r="M40" s="1" t="s">
-        <v>280</v>
-      </c>
-    </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A41" s="1" t="s">
-        <v>281</v>
-      </c>
-      <c r="B41" s="2">
+        <v>282</v>
+      </c>
+      <c r="N40" s="2"/>
+    </row>
+    <row r="41" spans="1:14" s="8" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="8" t="s">
+        <v>283</v>
+      </c>
+      <c r="B41" s="9">
+        <v>5</v>
+      </c>
+      <c r="C41" s="8" t="s">
+        <v>251</v>
+      </c>
+      <c r="D41" s="8" t="s">
+        <v>284</v>
+      </c>
+      <c r="E41" s="8" t="s">
+        <v>286</v>
+      </c>
+      <c r="F41" s="8" t="s">
+        <v>285</v>
+      </c>
+      <c r="G41" s="8" t="s">
+        <v>433</v>
+      </c>
+      <c r="H41" s="8" t="s">
+        <v>287</v>
+      </c>
+      <c r="I41" s="10">
+        <v>1206</v>
+      </c>
+      <c r="J41" s="11">
+        <v>0.05</v>
+      </c>
+      <c r="K41" s="9"/>
+      <c r="L41" s="9"/>
+      <c r="M41" s="8" t="s">
+        <v>288</v>
+      </c>
+      <c r="N41" s="9"/>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A42" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="B42" s="2">
         <v>1</v>
       </c>
-      <c r="C41" s="1" t="s">
-        <v>282</v>
-      </c>
-      <c r="D41" s="1" t="s">
-        <v>276</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="F41" s="1" t="s">
-        <v>283</v>
-      </c>
-      <c r="G41" s="1" t="s">
-        <v>284</v>
-      </c>
-      <c r="H41" s="1" t="s">
-        <v>285</v>
-      </c>
-      <c r="I41" s="3" t="s">
-        <v>418</v>
-      </c>
-      <c r="J41" s="4">
-        <v>0.01</v>
-      </c>
-      <c r="M41" s="1" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A42" s="1" t="s">
-        <v>287</v>
-      </c>
-      <c r="B42" s="2">
-        <v>5</v>
-      </c>
       <c r="C42" s="1" t="s">
-        <v>255</v>
+        <v>290</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>288</v>
+        <v>252</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>290</v>
+        <v>18</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>289</v>
+        <v>291</v>
+      </c>
+      <c r="G42" s="1" t="s">
+        <v>292</v>
       </c>
       <c r="H42" s="1" t="s">
-        <v>291</v>
-      </c>
-      <c r="I42" s="3">
-        <v>1206</v>
+        <v>293</v>
+      </c>
+      <c r="I42" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="J42" s="4">
+        <v>0.05</v>
       </c>
       <c r="M42" s="1" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
+        <v>294</v>
+      </c>
+      <c r="N42" s="2"/>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="B43" s="2">
         <v>1</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>256</v>
+        <v>272</v>
       </c>
       <c r="E43" s="1" t="s">
         <v>18</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="H43" s="1" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="I43" s="3" t="s">
-        <v>419</v>
+        <v>414</v>
       </c>
       <c r="J43" s="4">
-        <v>0.05</v>
+        <v>0.01</v>
+      </c>
+      <c r="K43" s="2" t="s">
+        <v>40</v>
       </c>
       <c r="M43" s="1" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
+        <v>300</v>
+      </c>
+      <c r="N43" s="2"/>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="B44" s="2">
         <v>1</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>18</v>
+        <v>246</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="G44" s="1" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="H44" s="1" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="I44" s="3" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
       <c r="J44" s="4">
         <v>0.01</v>
@@ -3850,36 +3969,37 @@
         <v>40</v>
       </c>
       <c r="M44" s="1" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
+        <v>306</v>
+      </c>
+      <c r="N44" s="2"/>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="B45" s="2">
         <v>1</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="G45" s="1" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="I45" s="3" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
       <c r="J45" s="4">
         <v>0.01</v>
@@ -3888,488 +4008,470 @@
         <v>40</v>
       </c>
       <c r="M45" s="1" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
+        <v>312</v>
+      </c>
+      <c r="N45" s="2"/>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="B46" s="2">
         <v>1</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>276</v>
+        <v>252</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="G46" s="1" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="I46" s="3" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="J46" s="4">
         <v>0.01</v>
       </c>
-      <c r="K46" s="2" t="s">
-        <v>40</v>
-      </c>
       <c r="M46" s="1" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
+        <v>318</v>
+      </c>
+      <c r="N46" s="2"/>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="B47" s="2">
         <v>1</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="G47" s="1" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="H47" s="1" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="I47" s="3" t="s">
-        <v>419</v>
+        <v>415</v>
       </c>
       <c r="J47" s="4">
         <v>0.01</v>
       </c>
       <c r="M47" s="1" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
+        <v>324</v>
+      </c>
+      <c r="N47" s="2"/>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="B48" s="2">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>250</v>
+        <v>18</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="G48" s="1" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="H48" s="1" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="I48" s="3" t="s">
-        <v>419</v>
+        <v>415</v>
       </c>
       <c r="J48" s="4">
         <v>0.01</v>
       </c>
       <c r="M48" s="1" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
+        <v>330</v>
+      </c>
+      <c r="N48" s="2"/>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="B49" s="2">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>256</v>
+        <v>333</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>18</v>
+        <v>336</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="G49" s="1" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="H49" s="1" t="s">
-        <v>333</v>
+        <v>337</v>
       </c>
       <c r="I49" s="3" t="s">
-        <v>419</v>
-      </c>
-      <c r="J49" s="4">
-        <v>0.01</v>
+        <v>338</v>
       </c>
       <c r="M49" s="1" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
+        <v>339</v>
+      </c>
+      <c r="N49" s="2"/>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>335</v>
+        <v>340</v>
       </c>
       <c r="B50" s="2">
         <v>1</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>336</v>
+        <v>341</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>340</v>
+        <v>345</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>338</v>
+        <v>343</v>
       </c>
       <c r="G50" s="1" t="s">
-        <v>339</v>
+        <v>344</v>
       </c>
       <c r="H50" s="1" t="s">
         <v>341</v>
       </c>
       <c r="I50" s="3" t="s">
-        <v>342</v>
+        <v>346</v>
       </c>
       <c r="M50" s="1" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
+        <v>347</v>
+      </c>
+      <c r="N50" s="2"/>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>344</v>
+        <v>348</v>
       </c>
       <c r="B51" s="2">
         <v>1</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>345</v>
+        <v>349</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>346</v>
+        <v>350</v>
       </c>
       <c r="E51" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="G51" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="H51" s="1" t="s">
         <v>349</v>
       </c>
-      <c r="F51" s="1" t="s">
-        <v>347</v>
-      </c>
-      <c r="G51" s="1" t="s">
-        <v>348</v>
-      </c>
-      <c r="H51" s="1" t="s">
-        <v>345</v>
-      </c>
       <c r="I51" s="3" t="s">
-        <v>350</v>
+        <v>354</v>
+      </c>
+      <c r="K51" s="2" t="s">
+        <v>355</v>
+      </c>
+      <c r="L51" s="2" t="s">
+        <v>356</v>
       </c>
       <c r="M51" s="1" t="s">
-        <v>351</v>
-      </c>
-    </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
+        <v>357</v>
+      </c>
+      <c r="N51" s="2"/>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>352</v>
+        <v>358</v>
       </c>
       <c r="B52" s="2">
         <v>1</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>354</v>
+        <v>360</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>357</v>
+        <v>363</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>355</v>
+        <v>361</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>356</v>
+        <v>362</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>353</v>
+        <v>364</v>
       </c>
       <c r="I52" s="3" t="s">
-        <v>358</v>
-      </c>
-      <c r="K52" s="2" t="s">
-        <v>359</v>
-      </c>
-      <c r="L52" s="2" t="s">
-        <v>360</v>
+        <v>365</v>
       </c>
       <c r="M52" s="1" t="s">
-        <v>361</v>
-      </c>
-    </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
+        <v>366</v>
+      </c>
+      <c r="N52" s="2"/>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>362</v>
+        <v>367</v>
       </c>
       <c r="B53" s="2">
         <v>1</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>364</v>
+        <v>369</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>367</v>
+        <v>372</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>365</v>
+        <v>370</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>366</v>
+        <v>371</v>
       </c>
       <c r="H53" s="1" t="s">
         <v>368</v>
       </c>
       <c r="I53" s="3" t="s">
-        <v>369</v>
+        <v>373</v>
+      </c>
+      <c r="K53" s="2" t="s">
+        <v>374</v>
+      </c>
+      <c r="L53" s="2" t="s">
+        <v>375</v>
       </c>
       <c r="M53" s="1" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
+        <v>376</v>
+      </c>
+      <c r="N53" s="2"/>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>371</v>
+        <v>377</v>
       </c>
       <c r="B54" s="2">
         <v>1</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>372</v>
+        <v>378</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>373</v>
+        <v>379</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>376</v>
+        <v>382</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>374</v>
+        <v>380</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>372</v>
-      </c>
-      <c r="I54" s="3" t="s">
-        <v>377</v>
-      </c>
-      <c r="K54" s="2" t="s">
         <v>378</v>
       </c>
-      <c r="L54" s="2" t="s">
-        <v>379</v>
-      </c>
       <c r="M54" s="1" t="s">
-        <v>380</v>
-      </c>
-    </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
+        <v>383</v>
+      </c>
+      <c r="N54" s="2"/>
+    </row>
+    <row r="55" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="B55" s="2">
         <v>1</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>386</v>
+        <v>126</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="G55" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="H55" s="1" t="s">
         <v>385</v>
       </c>
-      <c r="H55" s="1" t="s">
-        <v>382</v>
+      <c r="I55" s="3" t="s">
+        <v>389</v>
+      </c>
+      <c r="L55" s="2" t="s">
+        <v>390</v>
       </c>
       <c r="M55" s="1" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
+        <v>391</v>
+      </c>
+      <c r="N55" s="2"/>
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>388</v>
+        <v>392</v>
       </c>
       <c r="B56" s="2">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>390</v>
+        <v>394</v>
       </c>
       <c r="E56" s="1" t="s">
         <v>126</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>391</v>
+        <v>395</v>
       </c>
       <c r="G56" s="1" t="s">
-        <v>392</v>
+        <v>396</v>
       </c>
       <c r="H56" s="1" t="s">
-        <v>389</v>
+        <v>393</v>
       </c>
       <c r="I56" s="3" t="s">
-        <v>393</v>
-      </c>
-      <c r="L56" s="2" t="s">
-        <v>394</v>
+        <v>346</v>
       </c>
       <c r="M56" s="1" t="s">
-        <v>395</v>
-      </c>
-    </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
+        <v>397</v>
+      </c>
+      <c r="N56" s="2"/>
+    </row>
+    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="B57" s="2">
         <v>4</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="E57" s="1" t="s">
-        <v>126</v>
+        <v>403</v>
       </c>
       <c r="F57" s="1" t="s">
+        <v>401</v>
+      </c>
+      <c r="G57" s="1" t="s">
+        <v>402</v>
+      </c>
+      <c r="H57" s="1" t="s">
         <v>399</v>
       </c>
-      <c r="G57" s="1" t="s">
-        <v>400</v>
-      </c>
-      <c r="H57" s="1" t="s">
-        <v>397</v>
-      </c>
       <c r="I57" s="3" t="s">
-        <v>350</v>
+        <v>404</v>
       </c>
       <c r="M57" s="1" t="s">
-        <v>401</v>
-      </c>
-    </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A58" s="1" t="s">
-        <v>402</v>
-      </c>
-      <c r="B58" s="2">
-        <v>4</v>
-      </c>
-      <c r="C58" s="1" t="s">
-        <v>403</v>
-      </c>
-      <c r="D58" s="1" t="s">
-        <v>404</v>
-      </c>
-      <c r="E58" s="1" t="s">
+        <v>405</v>
+      </c>
+      <c r="N57" s="2"/>
+    </row>
+    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A58" s="12" t="s">
+        <v>406</v>
+      </c>
+      <c r="B58" s="13">
+        <v>1</v>
+      </c>
+      <c r="C58" s="12" t="s">
         <v>407</v>
       </c>
-      <c r="F58" s="1" t="s">
-        <v>405</v>
-      </c>
-      <c r="G58" s="1" t="s">
-        <v>406</v>
-      </c>
-      <c r="H58" s="1" t="s">
-        <v>403</v>
-      </c>
-      <c r="I58" s="3" t="s">
+      <c r="D58" s="12" t="s">
         <v>408</v>
       </c>
-      <c r="M58" s="1" t="s">
+      <c r="E58" s="12" t="s">
+        <v>411</v>
+      </c>
+      <c r="F58" s="12" t="s">
         <v>409</v>
       </c>
-    </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A59" s="1" t="s">
+      <c r="G58" s="12" t="s">
         <v>410</v>
       </c>
-      <c r="B59" s="2">
-        <v>1</v>
-      </c>
-      <c r="C59" s="1" t="s">
-        <v>411</v>
-      </c>
-      <c r="D59" s="1" t="s">
+      <c r="H58" s="12" t="s">
+        <v>407</v>
+      </c>
+      <c r="I58" s="14" t="s">
         <v>412</v>
       </c>
-      <c r="E59" s="1" t="s">
-        <v>415</v>
-      </c>
-      <c r="F59" s="1" t="s">
+      <c r="J58" s="13"/>
+      <c r="K58" s="13"/>
+      <c r="L58" s="13"/>
+      <c r="M58" s="12" t="s">
         <v>413</v>
       </c>
-      <c r="G59" s="1" t="s">
-        <v>414</v>
-      </c>
-      <c r="H59" s="1" t="s">
-        <v>411</v>
-      </c>
-      <c r="I59" s="3" t="s">
-        <v>416</v>
-      </c>
-      <c r="M59" s="1" t="s">
-        <v>417</v>
+      <c r="N58" s="2" t="s">
+        <v>435</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>